<commit_message>
data take 4 decimal place
</commit_message>
<xml_diff>
--- a/stock_returns_risk.xlsx
+++ b/stock_returns_risk.xlsx
@@ -452,10 +452,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>-0.01115680473191414</v>
+        <v>-0.0112</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0331878881921162</v>
+        <v>0.0332</v>
       </c>
     </row>
     <row r="3">
@@ -465,10 +465,10 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.04725592157478573</v>
+        <v>0.0473</v>
       </c>
       <c r="C3" t="n">
-        <v>0.07569331642213094</v>
+        <v>0.0757</v>
       </c>
     </row>
     <row r="4">
@@ -478,10 +478,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0355705697589721</v>
+        <v>0.0356</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1108835341965159</v>
+        <v>0.1109</v>
       </c>
     </row>
     <row r="5">
@@ -491,10 +491,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.5141519899424786</v>
+        <v>0.5142</v>
       </c>
       <c r="C5" t="n">
-        <v>0.8380421442799674</v>
+        <v>0.838</v>
       </c>
     </row>
     <row r="6">
@@ -504,10 +504,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.01402651055665103</v>
+        <v>0.014</v>
       </c>
       <c r="C6" t="n">
-        <v>0.09024931864907877</v>
+        <v>0.0902</v>
       </c>
     </row>
     <row r="7">
@@ -517,10 +517,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.01004121478127344</v>
+        <v>-0.01</v>
       </c>
       <c r="C7" t="n">
-        <v>0.04934867566020545</v>
+        <v>0.0493</v>
       </c>
     </row>
     <row r="8">
@@ -530,10 +530,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.05359635150934309</v>
+        <v>0.0536</v>
       </c>
       <c r="C8" t="n">
-        <v>0.1193907826527402</v>
+        <v>0.1194</v>
       </c>
     </row>
     <row r="9">
@@ -543,10 +543,10 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.01675870132897929</v>
+        <v>0.0168</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0542469738210138</v>
+        <v>0.0542</v>
       </c>
     </row>
     <row r="10">
@@ -556,10 +556,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.01861926461753061</v>
+        <v>0.0186</v>
       </c>
       <c r="C10" t="n">
-        <v>0.04078719348675861</v>
+        <v>0.0408</v>
       </c>
     </row>
     <row r="11">
@@ -569,10 +569,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0532436257687155</v>
+        <v>0.0532</v>
       </c>
       <c r="C11" t="n">
-        <v>0.1322383376398704</v>
+        <v>0.1322</v>
       </c>
     </row>
     <row r="12">
@@ -582,10 +582,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-0.002298764824702352</v>
+        <v>-0.0023</v>
       </c>
       <c r="C12" t="n">
-        <v>0.05726733924125114</v>
+        <v>0.0573</v>
       </c>
     </row>
     <row r="13">
@@ -595,10 +595,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.09724898091218466</v>
+        <v>0.09719999999999999</v>
       </c>
       <c r="C13" t="n">
-        <v>0.1242073408469463</v>
+        <v>0.1242</v>
       </c>
     </row>
     <row r="14">
@@ -608,10 +608,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.01052990793945452</v>
+        <v>0.0105</v>
       </c>
       <c r="C14" t="n">
-        <v>0.07987992422641019</v>
+        <v>0.0799</v>
       </c>
     </row>
     <row r="15">
@@ -621,10 +621,10 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.2182751942560942</v>
+        <v>0.2183</v>
       </c>
       <c r="C15" t="n">
-        <v>0.2649818644904063</v>
+        <v>0.265</v>
       </c>
     </row>
     <row r="16">
@@ -634,10 +634,10 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.005914085032652117</v>
+        <v>0.0059</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0357972232070545</v>
+        <v>0.0358</v>
       </c>
     </row>
     <row r="17">
@@ -647,10 +647,10 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.01225544163735872</v>
+        <v>0.0123</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0838087185693208</v>
+        <v>0.0838</v>
       </c>
     </row>
     <row r="18">
@@ -660,10 +660,10 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.212581845168545</v>
+        <v>0.2126</v>
       </c>
       <c r="C18" t="n">
-        <v>0.1855605901812327</v>
+        <v>0.1856</v>
       </c>
     </row>
     <row r="19">
@@ -673,10 +673,10 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>-0.009384517770331688</v>
+        <v>-0.0094</v>
       </c>
       <c r="C19" t="n">
-        <v>0.05514660334231174</v>
+        <v>0.0551</v>
       </c>
     </row>
     <row r="20">
@@ -686,10 +686,10 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>-0.04481161556580095</v>
+        <v>-0.0448</v>
       </c>
       <c r="C20" t="n">
-        <v>0.134050128580287</v>
+        <v>0.1341</v>
       </c>
     </row>
     <row r="21">
@@ -699,10 +699,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>-0.01832421549649403</v>
+        <v>-0.0183</v>
       </c>
       <c r="C21" t="n">
-        <v>0.2778279568338603</v>
+        <v>0.2778</v>
       </c>
     </row>
     <row r="22">
@@ -712,10 +712,10 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>-0.01308754568527219</v>
+        <v>-0.0131</v>
       </c>
       <c r="C22" t="n">
-        <v>0.1090366910818387</v>
+        <v>0.109</v>
       </c>
     </row>
     <row r="23">
@@ -725,10 +725,10 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>-0.07157730751898643</v>
+        <v>-0.0716</v>
       </c>
       <c r="C23" t="n">
-        <v>0.10863836773388</v>
+        <v>0.1086</v>
       </c>
     </row>
     <row r="24">
@@ -738,10 +738,10 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>-0.08720974229571171</v>
+        <v>-0.0872</v>
       </c>
       <c r="C24" t="n">
-        <v>0.07128315770299085</v>
+        <v>0.0713</v>
       </c>
     </row>
     <row r="25">
@@ -751,10 +751,10 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>0.002066814006729589</v>
+        <v>0.0021</v>
       </c>
       <c r="C25" t="n">
-        <v>0.1109898142489509</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="26">
@@ -764,10 +764,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.01437497220075793</v>
+        <v>0.0144</v>
       </c>
       <c r="C26" t="n">
-        <v>0.1194999840706898</v>
+        <v>0.1195</v>
       </c>
     </row>
     <row r="27">
@@ -777,10 +777,10 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.3975293114544349</v>
+        <v>0.3975</v>
       </c>
       <c r="C27" t="n">
-        <v>0.5821665514403882</v>
+        <v>0.5822000000000001</v>
       </c>
     </row>
     <row r="28">
@@ -790,10 +790,10 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>-0.01073993997877901</v>
+        <v>-0.0107</v>
       </c>
       <c r="C28" t="n">
-        <v>0.05704166975409821</v>
+        <v>0.057</v>
       </c>
     </row>
     <row r="29">
@@ -803,10 +803,10 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.01311900988103741</v>
+        <v>0.0131</v>
       </c>
       <c r="C29" t="n">
-        <v>0.05735711283697577</v>
+        <v>0.0574</v>
       </c>
     </row>
     <row r="30">
@@ -816,10 +816,10 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>-0.1500300024825274</v>
+        <v>-0.15</v>
       </c>
       <c r="C30" t="n">
-        <v>0.1003866690440173</v>
+        <v>0.1004</v>
       </c>
     </row>
     <row r="31">
@@ -829,10 +829,10 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.01377165215862131</v>
+        <v>0.0138</v>
       </c>
       <c r="C31" t="n">
-        <v>0.1399695894791362</v>
+        <v>0.14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>